<commit_message>
Prompt coach live test: plant known answers in GRC-1 to GRC-4
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sp6bbiPXfwDc65dz8hiGei
</commit_message>
<xml_diff>
--- a/prompt-coach/research/live-tests/fixtures/grc_rcm.xlsx
+++ b/prompt-coach/research/live-tests/fixtures/grc_rcm.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,6 +412,9 @@
       <c r="D1" t="str">
         <v>Frequency</v>
       </c>
+      <c r="E1" t="str">
+        <v>Key control</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -426,6 +429,9 @@
       <c r="D2" t="str">
         <v>Monthly</v>
       </c>
+      <c r="E2" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -440,6 +446,9 @@
       <c r="D3" t="str">
         <v>Quarterly</v>
       </c>
+      <c r="E3" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -454,6 +463,9 @@
       <c r="D4" t="str">
         <v/>
       </c>
+      <c r="E4" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -468,6 +480,9 @@
       <c r="D5" t="str">
         <v/>
       </c>
+      <c r="E5" t="str">
+        <v>No</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -482,10 +497,30 @@
       <c r="D6" t="str">
         <v>Monthly</v>
       </c>
+      <c r="E6" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>C-06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Inventory count</v>
+      </c>
+      <c r="C7" t="str">
+        <v>TBD</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Annual</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Yes</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>